<commit_message>
iterative optimisation to reduce time for solver to run with large numbers of boolean variables
</commit_message>
<xml_diff>
--- a/example/example/example_hansard.xlsx
+++ b/example/example/example_hansard.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28800" yWindow="600" windowWidth="38400" windowHeight="21000" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Participants" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,30 +13,23 @@
     <sheet name="Schedule" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -49,27 +43,12 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -82,20 +61,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -462,156 +437,156 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Person</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Assistant</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Assistant email</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Stacy Arnold</t>
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Seth Lang</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>StacyArnold@email.com</t>
+          <t>SethLang@email.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Stacy Arnold</t>
+          <t>Seth Lang</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>StacyArnold@email.com</t>
+          <t>SethLang@email.com</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Alexandra Flynn</t>
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Charles Brown</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AlexandraFlynn@email.com</t>
+          <t>CharlesBrown@email.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Alexandra Flynn</t>
+          <t>Charles Brown</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>AlexandraFlynn@email.com</t>
+          <t>CharlesBrown@email.com</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Tracy Tran</t>
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Mark Wilkins</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>TracyTran@email.com</t>
+          <t>MarkWilkins@email.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tracy Tran</t>
+          <t>Mark Wilkins</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>TracyTran@email.com</t>
+          <t>MarkWilkins@email.com</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Kathleen Salas</t>
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Susan Solis</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>KathleenSalas@email.com</t>
+          <t>SusanSolis@email.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Kathleen Salas</t>
+          <t>Susan Solis</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>KathleenSalas@email.com</t>
+          <t>SusanSolis@email.com</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Tyler Lewis</t>
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Sophia Scott</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TylerLewis@email.com</t>
+          <t>SophiaScott@email.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Tyler Lewis</t>
+          <t>Sophia Scott</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>TylerLewis@email.com</t>
+          <t>SophiaScott@email.com</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Tanya Thomas</t>
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Karen Miller</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TanyaThomas@email.com</t>
+          <t>KarenMiller@email.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Tanya Thomas</t>
+          <t>Karen Miller</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>TanyaThomas@email.com</t>
+          <t>KarenMiller@email.com</t>
         </is>
       </c>
     </row>
@@ -626,79 +601,85 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Period</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Start Date</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>End Date</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="5" t="n">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="n">
         <v>46082</v>
       </c>
-      <c r="C2" s="5" t="n">
+      <c r="C2" s="3" t="n">
         <v>46096</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B3" s="3" t="n">
         <v>46096</v>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="3" t="n">
         <v>46110</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="3" t="n">
         <v>46110</v>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="3" t="n">
         <v>46124</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="3" t="n">
         <v>46124</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="3" t="n">
         <v>46138</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="3" t="n">
         <v>46138</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="3" t="n">
         <v>46152</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>46152</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>46166</v>
       </c>
     </row>
   </sheetData>
@@ -712,45 +693,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Person</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Period 1</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Period 2</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Period 3</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Period 4</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Period 5</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Period 6</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Stacy Arnold</t>
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Seth Lang</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -768,11 +754,14 @@
       <c r="F2" t="n">
         <v>1</v>
       </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Alexandra Flynn</t>
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Charles Brown</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -790,18 +779,21 @@
       <c r="F3" t="n">
         <v>1</v>
       </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Tracy Tran</t>
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Mark Wilkins</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -812,11 +804,14 @@
       <c r="F4" t="n">
         <v>1</v>
       </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Kathleen Salas</t>
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Susan Solis</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -834,11 +829,14 @@
       <c r="F5" t="n">
         <v>1</v>
       </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Tyler Lewis</t>
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Sophia Scott</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -856,11 +854,14 @@
       <c r="F6" t="n">
         <v>1</v>
       </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Tanya Thomas</t>
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Karen Miller</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -876,6 +877,9 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -890,152 +894,265 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Person</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Period 1</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Period 2</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Period 3</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Period 4</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Period 5</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Period 6</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Stacy Arnold</t>
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Seth Lang</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Kathleen Salas</t>
+          <t>Charles Brown</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Alexandra Flynn</t>
+          <t>Sophia Scott</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tracy Tran</t>
+          <t>Mark Wilkins</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Susan Solis</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Karen Miller</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Charles Brown</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Alexandra Flynn</t>
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Charles Brown</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tyler Lewis</t>
+          <t>Seth Lang</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Stacy Arnold</t>
+          <t>Susan Solis</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Tanya Thomas</t>
+          <t>Karen Miller</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Mark Wilkins</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Sophia Scott</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Seth Lang</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Tracy Tran</t>
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Mark Wilkins</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Tanya Thomas</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>Sophia Scott</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Karen Miller</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Stacy Arnold</t>
+          <t>Seth Lang</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Charles Brown</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Susan Solis</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Sophia Scott</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Kathleen Salas</t>
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Susan Solis</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Stacy Arnold</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>Karen Miller</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Charles Brown</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Tyler Lewis</t>
+          <t>Sophia Scott</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Seth Lang</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Mark Wilkins</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Karen Miller</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Tyler Lewis</t>
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Sophia Scott</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alexandra Flynn</t>
+          <t>Mark Wilkins</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Tanya Thomas</t>
+          <t>Seth Lang</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Kathleen Salas</t>
+          <t>Susan Solis</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Karen Miller</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Charles Brown</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Mark Wilkins</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Tanya Thomas</t>
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Karen Miller</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Tracy Tran</t>
+          <t>Susan Solis</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Tyler Lewis</t>
+          <t>Mark Wilkins</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Alexandra Flynn</t>
+          <t>Charles Brown</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Sophia Scott</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Seth Lang</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Susan Solis</t>
         </is>
       </c>
     </row>

</xml_diff>